<commit_message>
Aggiornati roster e numeri di maglia delle squadre da file Excel
</commit_message>
<xml_diff>
--- a/documenti squadre e torneo 2026/LISTE SQUADRE NUMERI.xlsx
+++ b/documenti squadre e torneo 2026/LISTE SQUADRE NUMERI.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="313">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="432" uniqueCount="316">
   <si>
     <t>SQUADRA</t>
   </si>
@@ -30,7 +30,7 @@
     <t>DATA DI NASCITA</t>
   </si>
   <si>
-    <t>FC SBANFA</t>
+    <t xml:space="preserve">FC SBANFA X </t>
   </si>
   <si>
     <t>DE MARIO SARTOR</t>
@@ -93,7 +93,7 @@
     <t>RICCARDO</t>
   </si>
   <si>
-    <t>LA NUOVA BOTTE DEL RE</t>
+    <t>LA NUOVA BOTTE DEL RE X</t>
   </si>
   <si>
     <t>TALAMINI</t>
@@ -150,7 +150,7 @@
     <t>YURI</t>
   </si>
   <si>
-    <t>FAUSTI LEGNAMI - REAL MADRINK</t>
+    <t>FAUSTI LEGNAMI - REAL MADRINK X</t>
   </si>
   <si>
     <t>ZANELLA</t>
@@ -204,7 +204,7 @@
     <t>GIOSUE'</t>
   </si>
   <si>
-    <t>SBOCCA JUNIORS</t>
+    <t xml:space="preserve">SBOCCA JUNIORS x </t>
   </si>
   <si>
     <t>DE BONA</t>
@@ -291,7 +291,7 @@
     <t>IGOR</t>
   </si>
   <si>
-    <t>BAR LA COA</t>
+    <t>BAR LA COA X</t>
   </si>
   <si>
     <t>VECELLIO REANE</t>
@@ -378,7 +378,7 @@
     <t>SANTER</t>
   </si>
   <si>
-    <t>UNION CADORE VAJONT</t>
+    <t>UNION CADORE VAJONT X</t>
   </si>
   <si>
     <t>FRIGO TURCO</t>
@@ -453,7 +453,7 @@
     <t>MELCHIORI</t>
   </si>
   <si>
-    <t>BAR MURAZZI &amp; TORRE 2</t>
+    <t>BAR MURAZZI &amp; TORRE 2 X</t>
   </si>
   <si>
     <t>BAMOUSSA</t>
@@ -537,7 +537,7 @@
     <t>20/01/1986</t>
   </si>
   <si>
-    <t>CDH</t>
+    <t>CDH x</t>
   </si>
   <si>
     <t>CIOTTI</t>
@@ -546,6 +546,12 @@
     <t>25/08/2000</t>
   </si>
   <si>
+    <t xml:space="preserve">PANCIERA </t>
+  </si>
+  <si>
+    <t>FRANCO</t>
+  </si>
+  <si>
     <t>11/11/2001</t>
   </si>
   <si>
@@ -639,7 +645,7 @@
     <t>GIOELE</t>
   </si>
   <si>
-    <t>BAR SPRITZ&amp;COFFEE</t>
+    <t>BAR SPRITZ&amp;COFFEE X</t>
   </si>
   <si>
     <t>BUZZETTO</t>
@@ -672,7 +678,7 @@
     <t>VETTOREL</t>
   </si>
   <si>
-    <t>HR USIGNOLO</t>
+    <t>HR USIGNOLO X</t>
   </si>
   <si>
     <t>MEMIC</t>
@@ -693,36 +699,39 @@
     <t>DE SILVESTRO</t>
   </si>
   <si>
-    <t>SCREM</t>
+    <t xml:space="preserve">PAOLETTI </t>
+  </si>
+  <si>
+    <t xml:space="preserve">NICOLÒ </t>
+  </si>
+  <si>
+    <t>CORADAZZI</t>
+  </si>
+  <si>
+    <t>MONTAGNER</t>
+  </si>
+  <si>
+    <t>MANNEH</t>
+  </si>
+  <si>
+    <t>BABUCARR</t>
+  </si>
+  <si>
+    <t>PEDICINI</t>
+  </si>
+  <si>
+    <t>MASSIMILIANO</t>
+  </si>
+  <si>
+    <t>UNION SCP</t>
+  </si>
+  <si>
+    <t>DE DEMO</t>
   </si>
   <si>
     <t>MATTIA</t>
   </si>
   <si>
-    <t>CORADAZZI</t>
-  </si>
-  <si>
-    <t>MONTAGNER</t>
-  </si>
-  <si>
-    <t>MANNEH</t>
-  </si>
-  <si>
-    <t>BABUCARR</t>
-  </si>
-  <si>
-    <t>PEDICINI</t>
-  </si>
-  <si>
-    <t>MASSIMILIANO</t>
-  </si>
-  <si>
-    <t>UNION SCP</t>
-  </si>
-  <si>
-    <t>DE DEMO</t>
-  </si>
-  <si>
     <t>DE FINA</t>
   </si>
   <si>
@@ -750,7 +759,7 @@
     <t>ANTONY</t>
   </si>
   <si>
-    <t>CANTON n°4</t>
+    <t>CANTON n°4 x</t>
   </si>
   <si>
     <t>PASSUELLO</t>
@@ -786,7 +795,7 @@
     <t>FANTUZ</t>
   </si>
   <si>
-    <t>CALDART DE LOTTO</t>
+    <t>CALDART DE LOTTO X</t>
   </si>
   <si>
     <t>VESPIGNANI</t>
@@ -876,7 +885,7 @@
     <t>06/06/2003</t>
   </si>
   <si>
-    <t>DIAMA</t>
+    <t>DIAMA X</t>
   </si>
   <si>
     <t>SIBONJIC</t>
@@ -909,7 +918,7 @@
     <t>NIKOLAS</t>
   </si>
   <si>
-    <t>MOCRO TEAM</t>
+    <t>MOCRO TEAM X</t>
   </si>
   <si>
     <t>DAL FARRA</t>
@@ -961,7 +970,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="dd/MM/yyyy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -975,6 +984,10 @@
     <font>
       <b/>
       <color theme="1"/>
+      <name val="Arial Narrow"/>
+    </font>
+    <font>
+      <color rgb="FFFF00FF"/>
       <name val="Arial Narrow"/>
     </font>
   </fonts>
@@ -1004,7 +1017,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -1026,11 +1039,11 @@
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
+    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
     <xf borderId="0" fillId="2" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="2" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" vertical="center"/>
@@ -1038,11 +1051,23 @@
     <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1345,8 +1370,10 @@
       <c r="D3" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="8">
+      <c r="E3" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F3" s="7">
         <v>39084.0</v>
       </c>
       <c r="G3" s="1"/>
@@ -1378,8 +1405,8 @@
       <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="8">
+      <c r="E4" s="8"/>
+      <c r="F4" s="7">
         <v>39436.0</v>
       </c>
       <c r="G4" s="1"/>
@@ -1411,8 +1438,10 @@
       <c r="D5" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="8">
+      <c r="E5" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F5" s="7">
         <v>39720.0</v>
       </c>
       <c r="G5" s="1"/>
@@ -1444,8 +1473,8 @@
       <c r="D6" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E6" s="7"/>
-      <c r="F6" s="8">
+      <c r="E6" s="8"/>
+      <c r="F6" s="7">
         <v>39156.0</v>
       </c>
       <c r="G6" s="1"/>
@@ -1477,8 +1506,10 @@
       <c r="D7" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E7" s="7"/>
-      <c r="F7" s="8">
+      <c r="E7" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F7" s="7">
         <v>39621.0</v>
       </c>
       <c r="G7" s="1"/>
@@ -1510,8 +1541,10 @@
       <c r="D8" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E8" s="7"/>
-      <c r="F8" s="8">
+      <c r="E8" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F8" s="7">
         <v>39669.0</v>
       </c>
       <c r="G8" s="1"/>
@@ -1543,8 +1576,10 @@
       <c r="D9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E9" s="7"/>
-      <c r="F9" s="8">
+      <c r="E9" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F9" s="7">
         <v>39680.0</v>
       </c>
       <c r="G9" s="1"/>
@@ -1576,8 +1611,10 @@
       <c r="D10" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="E10" s="7"/>
-      <c r="F10" s="8">
+      <c r="E10" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F10" s="7">
         <v>39804.0</v>
       </c>
       <c r="G10" s="1"/>
@@ -1609,8 +1646,8 @@
       <c r="D11" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E11" s="7"/>
-      <c r="F11" s="8">
+      <c r="E11" s="8"/>
+      <c r="F11" s="7">
         <v>39819.0</v>
       </c>
       <c r="G11" s="1"/>
@@ -1642,8 +1679,8 @@
       <c r="D12" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="8">
+      <c r="E12" s="8"/>
+      <c r="F12" s="7">
         <v>39749.0</v>
       </c>
       <c r="G12" s="9"/>
@@ -1672,13 +1709,15 @@
       <c r="B13" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="10" t="s">
+      <c r="C13" s="11" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="10" t="s">
+      <c r="D13" s="11" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="11"/>
+      <c r="E13" s="11">
+        <v>1.0</v>
+      </c>
       <c r="F13" s="12">
         <v>34877.0</v>
       </c>
@@ -1705,13 +1744,15 @@
     </row>
     <row r="14">
       <c r="A14" s="1"/>
-      <c r="C14" s="10" t="s">
+      <c r="C14" s="11" t="s">
         <v>29</v>
       </c>
-      <c r="D14" s="10" t="s">
+      <c r="D14" s="11" t="s">
         <v>30</v>
       </c>
-      <c r="E14" s="11"/>
+      <c r="E14" s="11">
+        <v>6.0</v>
+      </c>
       <c r="F14" s="12">
         <v>37272.0</v>
       </c>
@@ -1738,13 +1779,15 @@
     </row>
     <row r="15">
       <c r="A15" s="1"/>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="10" t="s">
+      <c r="D15" s="11" t="s">
         <v>32</v>
       </c>
-      <c r="E15" s="11"/>
+      <c r="E15" s="11">
+        <v>10.0</v>
+      </c>
       <c r="F15" s="12">
         <v>35911.0</v>
       </c>
@@ -1771,13 +1814,15 @@
     </row>
     <row r="16">
       <c r="A16" s="1"/>
-      <c r="C16" s="10" t="s">
+      <c r="C16" s="11" t="s">
         <v>6</v>
       </c>
-      <c r="D16" s="10" t="s">
+      <c r="D16" s="11" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="11"/>
+      <c r="E16" s="11">
+        <v>4.0</v>
+      </c>
       <c r="F16" s="12">
         <v>36572.0</v>
       </c>
@@ -1804,13 +1849,15 @@
     </row>
     <row r="17">
       <c r="A17" s="1"/>
-      <c r="C17" s="10" t="s">
+      <c r="C17" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="D17" s="10" t="s">
+      <c r="D17" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="11"/>
+      <c r="E17" s="11">
+        <v>11.0</v>
+      </c>
       <c r="F17" s="12">
         <v>36764.0</v>
       </c>
@@ -1837,13 +1884,15 @@
     </row>
     <row r="18">
       <c r="A18" s="1"/>
-      <c r="C18" s="10" t="s">
+      <c r="C18" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="D18" s="10" t="s">
+      <c r="D18" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E18" s="11"/>
+      <c r="E18" s="11">
+        <v>3.0</v>
+      </c>
       <c r="F18" s="12">
         <v>39784.0</v>
       </c>
@@ -1870,13 +1919,15 @@
     </row>
     <row r="19">
       <c r="A19" s="1"/>
-      <c r="C19" s="10" t="s">
+      <c r="C19" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="D19" s="10" t="s">
+      <c r="D19" s="11" t="s">
         <v>38</v>
       </c>
-      <c r="E19" s="11"/>
+      <c r="E19" s="11">
+        <v>2.0</v>
+      </c>
       <c r="F19" s="12">
         <v>32921.0</v>
       </c>
@@ -1903,13 +1954,15 @@
     </row>
     <row r="20">
       <c r="A20" s="1"/>
-      <c r="C20" s="10" t="s">
+      <c r="C20" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="D20" s="10" t="s">
+      <c r="D20" s="11" t="s">
         <v>40</v>
       </c>
-      <c r="E20" s="11"/>
+      <c r="E20" s="11">
+        <v>7.0</v>
+      </c>
       <c r="F20" s="12">
         <v>39004.0</v>
       </c>
@@ -1936,13 +1989,15 @@
     </row>
     <row r="21">
       <c r="A21" s="1"/>
-      <c r="C21" s="10" t="s">
+      <c r="C21" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="D21" s="10" t="s">
+      <c r="D21" s="11" t="s">
         <v>42</v>
       </c>
-      <c r="E21" s="11"/>
+      <c r="E21" s="11">
+        <v>5.0</v>
+      </c>
       <c r="F21" s="12">
         <v>36110.0</v>
       </c>
@@ -1969,13 +2024,13 @@
     </row>
     <row r="22">
       <c r="A22" s="1"/>
-      <c r="C22" s="10" t="s">
+      <c r="C22" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="D22" s="10" t="s">
+      <c r="D22" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="E22" s="11"/>
+      <c r="E22" s="13"/>
       <c r="F22" s="12">
         <v>34690.0</v>
       </c>
@@ -2005,14 +2060,16 @@
       <c r="B23" s="6" t="s">
         <v>45</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="14" t="s">
         <v>47</v>
       </c>
-      <c r="E23" s="7"/>
-      <c r="F23" s="8">
+      <c r="E23" s="14">
+        <v>1.0</v>
+      </c>
+      <c r="F23" s="7">
         <v>38257.0</v>
       </c>
       <c r="G23" s="1"/>
@@ -2038,14 +2095,16 @@
     </row>
     <row r="24">
       <c r="A24" s="1"/>
-      <c r="C24" s="6" t="s">
+      <c r="C24" s="14" t="s">
         <v>48</v>
       </c>
-      <c r="D24" s="6" t="s">
+      <c r="D24" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="E24" s="7"/>
-      <c r="F24" s="8">
+      <c r="E24" s="14">
+        <v>8.0</v>
+      </c>
+      <c r="F24" s="7">
         <v>38996.0</v>
       </c>
       <c r="G24" s="1"/>
@@ -2071,14 +2130,16 @@
     </row>
     <row r="25">
       <c r="A25" s="1"/>
-      <c r="C25" s="6" t="s">
+      <c r="C25" s="14" t="s">
         <v>50</v>
       </c>
-      <c r="D25" s="6" t="s">
+      <c r="D25" s="14" t="s">
         <v>51</v>
       </c>
-      <c r="E25" s="7"/>
-      <c r="F25" s="8">
+      <c r="E25" s="14">
+        <v>2.0</v>
+      </c>
+      <c r="F25" s="7">
         <v>38621.0</v>
       </c>
       <c r="G25" s="1"/>
@@ -2104,14 +2165,16 @@
     </row>
     <row r="26">
       <c r="A26" s="1"/>
-      <c r="C26" s="6" t="s">
+      <c r="C26" s="14" t="s">
         <v>52</v>
       </c>
-      <c r="D26" s="6" t="s">
+      <c r="D26" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E26" s="7"/>
-      <c r="F26" s="8">
+      <c r="E26" s="14">
+        <v>5.0</v>
+      </c>
+      <c r="F26" s="7">
         <v>38808.0</v>
       </c>
       <c r="G26" s="1"/>
@@ -2137,14 +2200,16 @@
     </row>
     <row r="27">
       <c r="A27" s="1"/>
-      <c r="C27" s="6" t="s">
+      <c r="C27" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="D27" s="6" t="s">
+      <c r="D27" s="14" t="s">
         <v>55</v>
       </c>
-      <c r="E27" s="7"/>
-      <c r="F27" s="8">
+      <c r="E27" s="14">
+        <v>11.0</v>
+      </c>
+      <c r="F27" s="7">
         <v>39116.0</v>
       </c>
       <c r="G27" s="1"/>
@@ -2170,14 +2235,16 @@
     </row>
     <row r="28">
       <c r="A28" s="1"/>
-      <c r="C28" s="6" t="s">
+      <c r="C28" s="14" t="s">
         <v>56</v>
       </c>
-      <c r="D28" s="6" t="s">
+      <c r="D28" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="E28" s="7"/>
-      <c r="F28" s="8">
+      <c r="E28" s="14">
+        <v>3.0</v>
+      </c>
+      <c r="F28" s="7">
         <v>38463.0</v>
       </c>
       <c r="G28" s="1"/>
@@ -2203,14 +2270,16 @@
     </row>
     <row r="29">
       <c r="A29" s="1"/>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="6" t="s">
+      <c r="D29" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="7"/>
-      <c r="F29" s="8">
+      <c r="E29" s="14">
+        <v>10.0</v>
+      </c>
+      <c r="F29" s="7">
         <v>39167.0</v>
       </c>
       <c r="G29" s="1"/>
@@ -2236,14 +2305,16 @@
     </row>
     <row r="30">
       <c r="A30" s="1"/>
-      <c r="C30" s="6" t="s">
+      <c r="C30" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="D30" s="6" t="s">
+      <c r="D30" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="E30" s="7"/>
-      <c r="F30" s="8">
+      <c r="E30" s="14">
+        <v>7.0</v>
+      </c>
+      <c r="F30" s="7">
         <v>38958.0</v>
       </c>
       <c r="G30" s="1"/>
@@ -2269,14 +2340,16 @@
     </row>
     <row r="31">
       <c r="A31" s="1"/>
-      <c r="C31" s="6" t="s">
+      <c r="C31" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="D31" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="E31" s="7"/>
-      <c r="F31" s="8">
+      <c r="E31" s="14">
+        <v>99.0</v>
+      </c>
+      <c r="F31" s="7">
         <v>36720.0</v>
       </c>
       <c r="G31" s="1"/>
@@ -2302,14 +2375,16 @@
     </row>
     <row r="32">
       <c r="A32" s="1"/>
-      <c r="C32" s="6" t="s">
+      <c r="C32" s="14" t="s">
         <v>61</v>
       </c>
-      <c r="D32" s="6" t="s">
+      <c r="D32" s="14" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="7"/>
-      <c r="F32" s="8">
+      <c r="E32" s="14">
+        <v>9.0</v>
+      </c>
+      <c r="F32" s="7">
         <v>37557.0</v>
       </c>
       <c r="G32" s="1"/>
@@ -2338,13 +2413,15 @@
       <c r="B33" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="11" t="s">
         <v>64</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="E33" s="11"/>
+      <c r="E33" s="11">
+        <v>10.0</v>
+      </c>
       <c r="F33" s="12">
         <v>36265.0</v>
       </c>
@@ -2371,13 +2448,15 @@
     </row>
     <row r="34">
       <c r="A34" s="1"/>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="11" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="E34" s="11"/>
+      <c r="E34" s="11">
+        <v>9.0</v>
+      </c>
       <c r="F34" s="12">
         <v>36040.0</v>
       </c>
@@ -2404,13 +2483,15 @@
     </row>
     <row r="35">
       <c r="A35" s="1"/>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="11" t="s">
         <v>67</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E35" s="11"/>
+      <c r="E35" s="11">
+        <v>11.0</v>
+      </c>
       <c r="F35" s="12">
         <v>35782.0</v>
       </c>
@@ -2437,13 +2518,15 @@
     </row>
     <row r="36">
       <c r="A36" s="1"/>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="E36" s="11"/>
+      <c r="E36" s="11">
+        <v>1.0</v>
+      </c>
       <c r="F36" s="12">
         <v>37047.0</v>
       </c>
@@ -2470,13 +2553,15 @@
     </row>
     <row r="37">
       <c r="A37" s="1"/>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="11" t="s">
         <v>70</v>
       </c>
-      <c r="E37" s="11"/>
+      <c r="E37" s="11">
+        <v>8.0</v>
+      </c>
       <c r="F37" s="12">
         <v>36533.0</v>
       </c>
@@ -2503,13 +2588,15 @@
     </row>
     <row r="38">
       <c r="A38" s="1"/>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="11" t="s">
         <v>72</v>
       </c>
-      <c r="E38" s="11"/>
+      <c r="E38" s="11">
+        <v>7.0</v>
+      </c>
       <c r="F38" s="12">
         <v>35369.0</v>
       </c>
@@ -2536,13 +2623,15 @@
     </row>
     <row r="39">
       <c r="A39" s="1"/>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="11" t="s">
         <v>73</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="E39" s="11"/>
+      <c r="E39" s="11">
+        <v>2.0</v>
+      </c>
       <c r="F39" s="12">
         <v>36767.0</v>
       </c>
@@ -2569,13 +2658,15 @@
     </row>
     <row r="40">
       <c r="A40" s="1"/>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="11" t="s">
         <v>74</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="E40" s="11"/>
+      <c r="E40" s="11">
+        <v>3.0</v>
+      </c>
       <c r="F40" s="12">
         <v>39623.0</v>
       </c>
@@ -2602,13 +2693,13 @@
     </row>
     <row r="41">
       <c r="A41" s="1"/>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="11" t="s">
         <v>75</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="11" t="s">
         <v>55</v>
       </c>
-      <c r="E41" s="11"/>
+      <c r="E41" s="13"/>
       <c r="F41" s="12">
         <v>32862.0</v>
       </c>
@@ -2635,13 +2726,15 @@
     </row>
     <row r="42">
       <c r="A42" s="1"/>
-      <c r="C42" s="10" t="s">
+      <c r="C42" s="11" t="s">
         <v>76</v>
       </c>
-      <c r="D42" s="10" t="s">
+      <c r="D42" s="11" t="s">
         <v>77</v>
       </c>
-      <c r="E42" s="11"/>
+      <c r="E42" s="11">
+        <v>6.0</v>
+      </c>
       <c r="F42" s="12">
         <v>35441.0</v>
       </c>
@@ -2671,14 +2764,14 @@
       <c r="B43" s="6" t="s">
         <v>78</v>
       </c>
-      <c r="C43" s="6" t="s">
+      <c r="C43" s="14" t="s">
         <v>79</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="D43" s="14" t="s">
         <v>17</v>
       </c>
-      <c r="E43" s="7"/>
-      <c r="F43" s="8">
+      <c r="E43" s="15"/>
+      <c r="F43" s="7">
         <v>38383.0</v>
       </c>
       <c r="G43" s="1"/>
@@ -2704,14 +2797,16 @@
     </row>
     <row r="44">
       <c r="A44" s="1"/>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="14" t="s">
         <v>80</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="D44" s="14" t="s">
         <v>81</v>
       </c>
-      <c r="E44" s="7"/>
-      <c r="F44" s="8">
+      <c r="E44" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="F44" s="7">
         <v>38305.0</v>
       </c>
       <c r="G44" s="1"/>
@@ -2737,14 +2832,16 @@
     </row>
     <row r="45">
       <c r="A45" s="1"/>
-      <c r="C45" s="6" t="s">
+      <c r="C45" s="14" t="s">
         <v>82</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="D45" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E45" s="7"/>
-      <c r="F45" s="8">
+      <c r="E45" s="14">
+        <v>3.0</v>
+      </c>
+      <c r="F45" s="7">
         <v>37812.0</v>
       </c>
       <c r="G45" s="1"/>
@@ -2770,14 +2867,16 @@
     </row>
     <row r="46">
       <c r="A46" s="1"/>
-      <c r="C46" s="6" t="s">
+      <c r="C46" s="14" t="s">
         <v>83</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="D46" s="14" t="s">
         <v>84</v>
       </c>
-      <c r="E46" s="7"/>
-      <c r="F46" s="8">
+      <c r="E46" s="14">
+        <v>9.0</v>
+      </c>
+      <c r="F46" s="7">
         <v>37812.0</v>
       </c>
       <c r="G46" s="1"/>
@@ -2803,14 +2902,16 @@
     </row>
     <row r="47">
       <c r="A47" s="1"/>
-      <c r="C47" s="6" t="s">
+      <c r="C47" s="14" t="s">
         <v>68</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="D47" s="14" t="s">
         <v>57</v>
       </c>
-      <c r="E47" s="7"/>
-      <c r="F47" s="8">
+      <c r="E47" s="14">
+        <v>16.0</v>
+      </c>
+      <c r="F47" s="7">
         <v>38246.0</v>
       </c>
       <c r="G47" s="1"/>
@@ -2836,14 +2937,16 @@
     </row>
     <row r="48">
       <c r="A48" s="1"/>
-      <c r="C48" s="6" t="s">
+      <c r="C48" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D48" s="6" t="s">
+      <c r="D48" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="E48" s="7"/>
-      <c r="F48" s="8">
+      <c r="E48" s="14">
+        <v>12.0</v>
+      </c>
+      <c r="F48" s="7">
         <v>38068.0</v>
       </c>
       <c r="G48" s="1"/>
@@ -2869,14 +2972,16 @@
     </row>
     <row r="49">
       <c r="A49" s="1"/>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="14" t="s">
         <v>85</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="14" t="s">
         <v>86</v>
       </c>
-      <c r="E49" s="7"/>
-      <c r="F49" s="8">
+      <c r="E49" s="14">
+        <v>11.0</v>
+      </c>
+      <c r="F49" s="7">
         <v>38950.0</v>
       </c>
       <c r="G49" s="1"/>
@@ -2902,14 +3007,16 @@
     </row>
     <row r="50">
       <c r="A50" s="1"/>
-      <c r="C50" s="6" t="s">
+      <c r="C50" s="14" t="s">
         <v>87</v>
       </c>
-      <c r="D50" s="6" t="s">
+      <c r="D50" s="14" t="s">
         <v>88</v>
       </c>
-      <c r="E50" s="7"/>
-      <c r="F50" s="8">
+      <c r="E50" s="14">
+        <v>19.0</v>
+      </c>
+      <c r="F50" s="7">
         <v>38041.0</v>
       </c>
       <c r="G50" s="1"/>
@@ -2935,14 +3042,16 @@
     </row>
     <row r="51">
       <c r="A51" s="1"/>
-      <c r="C51" s="6" t="s">
+      <c r="C51" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="D51" s="6" t="s">
+      <c r="D51" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E51" s="7"/>
-      <c r="F51" s="8">
+      <c r="E51" s="14">
+        <v>20.0</v>
+      </c>
+      <c r="F51" s="7">
         <v>38552.0</v>
       </c>
       <c r="G51" s="1"/>
@@ -2968,14 +3077,16 @@
     </row>
     <row r="52">
       <c r="A52" s="1"/>
-      <c r="C52" s="6" t="s">
+      <c r="C52" s="14" t="s">
         <v>90</v>
       </c>
-      <c r="D52" s="6" t="s">
+      <c r="D52" s="14" t="s">
         <v>91</v>
       </c>
-      <c r="E52" s="7"/>
-      <c r="F52" s="8">
+      <c r="E52" s="14">
+        <v>18.0</v>
+      </c>
+      <c r="F52" s="7">
         <v>31357.0</v>
       </c>
       <c r="G52" s="1"/>
@@ -3010,7 +3121,9 @@
       <c r="D53" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E53" s="11"/>
+      <c r="E53" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F53" s="12">
         <v>37962.0</v>
       </c>
@@ -3043,7 +3156,9 @@
       <c r="D54" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="E54" s="11"/>
+      <c r="E54" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F54" s="12">
         <v>36607.0</v>
       </c>
@@ -3076,7 +3191,9 @@
       <c r="D55" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E55" s="11"/>
+      <c r="E55" s="10">
+        <v>20.0</v>
+      </c>
       <c r="F55" s="12">
         <v>36080.0</v>
       </c>
@@ -3109,7 +3226,9 @@
       <c r="D56" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E56" s="11"/>
+      <c r="E56" s="10">
+        <v>21.0</v>
+      </c>
       <c r="F56" s="12">
         <v>38015.0</v>
       </c>
@@ -3142,7 +3261,9 @@
       <c r="D57" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E57" s="11"/>
+      <c r="E57" s="10">
+        <v>2.0</v>
+      </c>
       <c r="F57" s="12">
         <v>39460.0</v>
       </c>
@@ -3175,7 +3296,9 @@
       <c r="D58" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="E58" s="11"/>
+      <c r="E58" s="10">
+        <v>11.0</v>
+      </c>
       <c r="F58" s="12">
         <v>39636.0</v>
       </c>
@@ -3208,7 +3331,9 @@
       <c r="D59" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="E59" s="11"/>
+      <c r="E59" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F59" s="12">
         <v>39340.0</v>
       </c>
@@ -3241,7 +3366,9 @@
       <c r="D60" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="E60" s="11"/>
+      <c r="E60" s="10">
+        <v>4.0</v>
+      </c>
       <c r="F60" s="12">
         <v>38637.0</v>
       </c>
@@ -3274,7 +3401,9 @@
       <c r="D61" s="10" t="s">
         <v>106</v>
       </c>
-      <c r="E61" s="11"/>
+      <c r="E61" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F61" s="12">
         <v>38872.0</v>
       </c>
@@ -3310,8 +3439,10 @@
       <c r="D62" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E62" s="7"/>
-      <c r="F62" s="8">
+      <c r="E62" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F62" s="7">
         <v>37818.0</v>
       </c>
       <c r="G62" s="1"/>
@@ -3343,8 +3474,10 @@
       <c r="D63" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E63" s="7"/>
-      <c r="F63" s="8">
+      <c r="E63" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="F63" s="7">
         <v>36516.0</v>
       </c>
       <c r="G63" s="1"/>
@@ -3376,8 +3509,10 @@
       <c r="D64" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E64" s="7"/>
-      <c r="F64" s="8">
+      <c r="E64" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F64" s="7">
         <v>37384.0</v>
       </c>
       <c r="G64" s="1"/>
@@ -3409,8 +3544,10 @@
       <c r="D65" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E65" s="7"/>
-      <c r="F65" s="8">
+      <c r="E65" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F65" s="7">
         <v>36381.0</v>
       </c>
       <c r="G65" s="1"/>
@@ -3442,8 +3579,10 @@
       <c r="D66" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E66" s="7"/>
-      <c r="F66" s="8">
+      <c r="E66" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F66" s="7">
         <v>35875.0</v>
       </c>
       <c r="G66" s="1"/>
@@ -3475,8 +3614,10 @@
       <c r="D67" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E67" s="7"/>
-      <c r="F67" s="8">
+      <c r="E67" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F67" s="7">
         <v>35888.0</v>
       </c>
       <c r="G67" s="1"/>
@@ -3508,8 +3649,10 @@
       <c r="D68" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="E68" s="7"/>
-      <c r="F68" s="8">
+      <c r="E68" s="6">
+        <v>75.0</v>
+      </c>
+      <c r="F68" s="7">
         <v>36452.0</v>
       </c>
       <c r="G68" s="1"/>
@@ -3541,8 +3684,10 @@
       <c r="D69" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E69" s="7"/>
-      <c r="F69" s="8">
+      <c r="E69" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F69" s="7">
         <v>35879.0</v>
       </c>
       <c r="G69" s="1"/>
@@ -3574,8 +3719,10 @@
       <c r="D70" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E70" s="7"/>
-      <c r="F70" s="8">
+      <c r="E70" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F70" s="7">
         <v>36345.0</v>
       </c>
       <c r="G70" s="1"/>
@@ -3607,8 +3754,10 @@
       <c r="D71" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E71" s="7"/>
-      <c r="F71" s="8">
+      <c r="E71" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F71" s="7">
         <v>36882.0</v>
       </c>
       <c r="G71" s="1"/>
@@ -3643,7 +3792,9 @@
       <c r="D72" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="E72" s="11"/>
+      <c r="E72" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F72" s="12">
         <v>35927.0</v>
       </c>
@@ -3676,7 +3827,9 @@
       <c r="D73" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E73" s="11"/>
+      <c r="E73" s="10">
+        <v>2.0</v>
+      </c>
       <c r="F73" s="12">
         <v>37942.0</v>
       </c>
@@ -3709,7 +3862,9 @@
       <c r="D74" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E74" s="11"/>
+      <c r="E74" s="10">
+        <v>3.0</v>
+      </c>
       <c r="F74" s="12">
         <v>38933.0</v>
       </c>
@@ -3742,7 +3897,9 @@
       <c r="D75" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="E75" s="11"/>
+      <c r="E75" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F75" s="12">
         <v>37893.0</v>
       </c>
@@ -3775,7 +3932,9 @@
       <c r="D76" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E76" s="11"/>
+      <c r="E76" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F76" s="12">
         <v>39359.0</v>
       </c>
@@ -3808,7 +3967,9 @@
       <c r="D77" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E77" s="11"/>
+      <c r="E77" s="10">
+        <v>11.0</v>
+      </c>
       <c r="F77" s="12">
         <v>37775.0</v>
       </c>
@@ -3841,7 +4002,9 @@
       <c r="D78" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="E78" s="11"/>
+      <c r="E78" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F78" s="12">
         <v>38821.0</v>
       </c>
@@ -3874,7 +4037,9 @@
       <c r="D79" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E79" s="11"/>
+      <c r="E79" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F79" s="12">
         <v>30965.0</v>
       </c>
@@ -3907,7 +4072,9 @@
       <c r="D80" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="E80" s="11"/>
+      <c r="E80" s="10">
+        <v>45.0</v>
+      </c>
       <c r="F80" s="12">
         <v>36769.0</v>
       </c>
@@ -3940,7 +4107,9 @@
       <c r="D81" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E81" s="11"/>
+      <c r="E81" s="10">
+        <v>98.0</v>
+      </c>
       <c r="F81" s="12">
         <v>39027.0</v>
       </c>
@@ -3976,8 +4145,10 @@
       <c r="D82" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E82" s="6"/>
-      <c r="F82" s="8">
+      <c r="E82" s="6">
+        <v>36.0</v>
+      </c>
+      <c r="F82" s="7">
         <v>36374.0</v>
       </c>
       <c r="G82" s="1"/>
@@ -4009,8 +4180,10 @@
       <c r="D83" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="E83" s="6"/>
-      <c r="F83" s="8">
+      <c r="E83" s="6">
+        <v>44.0</v>
+      </c>
+      <c r="F83" s="7">
         <v>35284.0</v>
       </c>
       <c r="G83" s="1"/>
@@ -4042,8 +4215,10 @@
       <c r="D84" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="E84" s="6"/>
-      <c r="F84" s="8">
+      <c r="E84" s="6">
+        <v>77.0</v>
+      </c>
+      <c r="F84" s="7">
         <v>34985.0</v>
       </c>
       <c r="G84" s="1"/>
@@ -4075,8 +4250,10 @@
       <c r="D85" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E85" s="6"/>
-      <c r="F85" s="8">
+      <c r="E85" s="6">
+        <v>14.0</v>
+      </c>
+      <c r="F85" s="7">
         <v>33856.0</v>
       </c>
       <c r="G85" s="1"/>
@@ -4108,8 +4285,10 @@
       <c r="D86" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E86" s="6"/>
-      <c r="F86" s="8">
+      <c r="E86" s="6">
+        <v>71.0</v>
+      </c>
+      <c r="F86" s="7">
         <v>35184.0</v>
       </c>
       <c r="G86" s="1"/>
@@ -4141,8 +4320,10 @@
       <c r="D87" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="E87" s="6"/>
-      <c r="F87" s="8">
+      <c r="E87" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F87" s="7">
         <v>37005.0</v>
       </c>
       <c r="G87" s="1"/>
@@ -4174,8 +4355,10 @@
       <c r="D88" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E88" s="6"/>
-      <c r="F88" s="8">
+      <c r="E88" s="6">
+        <v>74.0</v>
+      </c>
+      <c r="F88" s="7">
         <v>35254.0</v>
       </c>
       <c r="G88" s="1"/>
@@ -4207,8 +4390,10 @@
       <c r="D89" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="E89" s="6"/>
-      <c r="F89" s="8">
+      <c r="E89" s="6">
+        <v>0.0</v>
+      </c>
+      <c r="F89" s="7">
         <v>36781.0</v>
       </c>
       <c r="G89" s="1"/>
@@ -4240,8 +4425,10 @@
       <c r="D90" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E90" s="6"/>
-      <c r="F90" s="8">
+      <c r="E90" s="6">
+        <v>90.0</v>
+      </c>
+      <c r="F90" s="7">
         <v>34830.0</v>
       </c>
       <c r="G90" s="1"/>
@@ -4276,7 +4463,9 @@
       <c r="D91" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E91" s="11"/>
+      <c r="E91" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F91" s="12" t="s">
         <v>149</v>
       </c>
@@ -4309,7 +4498,9 @@
       <c r="D92" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="E92" s="11"/>
+      <c r="E92" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F92" s="12" t="s">
         <v>151</v>
       </c>
@@ -4342,7 +4533,9 @@
       <c r="D93" s="10" t="s">
         <v>153</v>
       </c>
-      <c r="E93" s="11"/>
+      <c r="E93" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F93" s="12" t="s">
         <v>154</v>
       </c>
@@ -4375,7 +4568,9 @@
       <c r="D94" s="10" t="s">
         <v>156</v>
       </c>
-      <c r="E94" s="11"/>
+      <c r="E94" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F94" s="12" t="s">
         <v>157</v>
       </c>
@@ -4408,7 +4603,9 @@
       <c r="D95" s="10" t="s">
         <v>159</v>
       </c>
-      <c r="E95" s="11"/>
+      <c r="E95" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F95" s="12" t="s">
         <v>160</v>
       </c>
@@ -4441,7 +4638,9 @@
       <c r="D96" s="10" t="s">
         <v>162</v>
       </c>
-      <c r="E96" s="11"/>
+      <c r="E96" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F96" s="12" t="s">
         <v>163</v>
       </c>
@@ -4474,7 +4673,7 @@
       <c r="D97" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="E97" s="11"/>
+      <c r="E97" s="16"/>
       <c r="F97" s="12" t="s">
         <v>165</v>
       </c>
@@ -4507,7 +4706,7 @@
       <c r="D98" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="E98" s="11"/>
+      <c r="E98" s="16"/>
       <c r="F98" s="12" t="s">
         <v>168</v>
       </c>
@@ -4540,7 +4739,7 @@
       <c r="D99" s="10" t="s">
         <v>170</v>
       </c>
-      <c r="E99" s="11"/>
+      <c r="E99" s="16"/>
       <c r="F99" s="12" t="s">
         <v>171</v>
       </c>
@@ -4573,7 +4772,7 @@
       <c r="D100" s="10" t="s">
         <v>148</v>
       </c>
-      <c r="E100" s="11"/>
+      <c r="E100" s="16"/>
       <c r="F100" s="12" t="s">
         <v>173</v>
       </c>
@@ -4609,8 +4808,10 @@
       <c r="D101" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E101" s="6"/>
-      <c r="F101" s="8" t="s">
+      <c r="E101" s="6">
+        <v>36.0</v>
+      </c>
+      <c r="F101" s="7" t="s">
         <v>176</v>
       </c>
       <c r="G101" s="1"/>
@@ -4637,14 +4838,16 @@
     <row r="102">
       <c r="A102" s="1"/>
       <c r="C102" s="6" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="D102" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="E102" s="6"/>
-      <c r="F102" s="8" t="s">
-        <v>177</v>
+        <v>178</v>
+      </c>
+      <c r="E102" s="6">
+        <v>90.0</v>
+      </c>
+      <c r="F102" s="7" t="s">
+        <v>179</v>
       </c>
       <c r="G102" s="1"/>
       <c r="H102" s="1"/>
@@ -4670,14 +4873,16 @@
     <row r="103">
       <c r="A103" s="1"/>
       <c r="C103" s="6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D103" s="6" t="s">
-        <v>179</v>
-      </c>
-      <c r="E103" s="6"/>
-      <c r="F103" s="8" t="s">
-        <v>180</v>
+        <v>181</v>
+      </c>
+      <c r="E103" s="6">
+        <v>17.0</v>
+      </c>
+      <c r="F103" s="7" t="s">
+        <v>182</v>
       </c>
       <c r="G103" s="1"/>
       <c r="H103" s="1"/>
@@ -4706,11 +4911,13 @@
         <v>34</v>
       </c>
       <c r="D104" s="6" t="s">
-        <v>181</v>
-      </c>
-      <c r="E104" s="6"/>
-      <c r="F104" s="8" t="s">
-        <v>182</v>
+        <v>183</v>
+      </c>
+      <c r="E104" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F104" s="7" t="s">
+        <v>184</v>
       </c>
       <c r="G104" s="1"/>
       <c r="H104" s="1"/>
@@ -4736,14 +4943,16 @@
     <row r="105">
       <c r="A105" s="1"/>
       <c r="C105" s="6" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D105" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E105" s="6"/>
-      <c r="F105" s="8" t="s">
-        <v>184</v>
+      <c r="E105" s="6">
+        <v>18.0</v>
+      </c>
+      <c r="F105" s="7" t="s">
+        <v>186</v>
       </c>
       <c r="G105" s="1"/>
       <c r="H105" s="1"/>
@@ -4774,9 +4983,11 @@
       <c r="D106" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E106" s="6"/>
-      <c r="F106" s="8" t="s">
-        <v>185</v>
+      <c r="E106" s="6">
+        <v>69.0</v>
+      </c>
+      <c r="F106" s="7" t="s">
+        <v>187</v>
       </c>
       <c r="G106" s="1"/>
       <c r="H106" s="1"/>
@@ -4802,14 +5013,16 @@
     <row r="107">
       <c r="A107" s="1"/>
       <c r="C107" s="6" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="D107" s="6" t="s">
-        <v>187</v>
-      </c>
-      <c r="E107" s="6"/>
-      <c r="F107" s="8" t="s">
-        <v>188</v>
+        <v>189</v>
+      </c>
+      <c r="E107" s="6">
+        <v>99.0</v>
+      </c>
+      <c r="F107" s="7" t="s">
+        <v>190</v>
       </c>
       <c r="G107" s="1"/>
       <c r="H107" s="1"/>
@@ -4835,14 +5048,16 @@
     <row r="108">
       <c r="A108" s="1"/>
       <c r="C108" s="6" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="D108" s="6" t="s">
         <v>84</v>
       </c>
-      <c r="E108" s="6"/>
-      <c r="F108" s="8" t="s">
-        <v>190</v>
+      <c r="E108" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F108" s="7" t="s">
+        <v>192</v>
       </c>
       <c r="G108" s="1"/>
       <c r="H108" s="1"/>
@@ -4868,15 +5083,17 @@
     <row r="109">
       <c r="A109" s="1"/>
       <c r="B109" s="10" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="C109" s="10" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="D109" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E109" s="11"/>
+      <c r="E109" s="10">
+        <v>11.0</v>
+      </c>
       <c r="F109" s="12">
         <v>39624.0</v>
       </c>
@@ -4904,12 +5121,14 @@
     <row r="110">
       <c r="A110" s="1"/>
       <c r="C110" s="10" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D110" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="E110" s="11"/>
+      <c r="E110" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F110" s="12">
         <v>40354.0</v>
       </c>
@@ -4942,7 +5161,9 @@
       <c r="D111" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="E111" s="11"/>
+      <c r="E111" s="10">
+        <v>2.0</v>
+      </c>
       <c r="F111" s="12">
         <v>38353.0</v>
       </c>
@@ -4970,12 +5191,14 @@
     <row r="112">
       <c r="A112" s="1"/>
       <c r="C112" s="10" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="D112" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="E112" s="11"/>
+        <v>197</v>
+      </c>
+      <c r="E112" s="10">
+        <v>4.0</v>
+      </c>
       <c r="F112" s="12">
         <v>39332.0</v>
       </c>
@@ -5003,12 +5226,14 @@
     <row r="113">
       <c r="A113" s="1"/>
       <c r="C113" s="10" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D113" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="E113" s="11"/>
+        <v>199</v>
+      </c>
+      <c r="E113" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F113" s="12">
         <v>38841.0</v>
       </c>
@@ -5036,12 +5261,14 @@
     <row r="114">
       <c r="A114" s="1"/>
       <c r="C114" s="10" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="D114" s="10" t="s">
-        <v>199</v>
-      </c>
-      <c r="E114" s="11"/>
+        <v>201</v>
+      </c>
+      <c r="E114" s="10">
+        <v>7.0</v>
+      </c>
       <c r="F114" s="12">
         <v>38520.0</v>
       </c>
@@ -5069,12 +5296,14 @@
     <row r="115">
       <c r="A115" s="1"/>
       <c r="C115" s="10" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D115" s="10" t="s">
-        <v>201</v>
-      </c>
-      <c r="E115" s="11"/>
+        <v>203</v>
+      </c>
+      <c r="E115" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F115" s="12">
         <v>39596.0</v>
       </c>
@@ -5102,12 +5331,14 @@
     <row r="116">
       <c r="A116" s="1"/>
       <c r="C116" s="10" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="D116" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="E116" s="11"/>
+      <c r="E116" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F116" s="12">
         <v>39578.0</v>
       </c>
@@ -5135,12 +5366,14 @@
     <row r="117">
       <c r="A117" s="1"/>
       <c r="C117" s="10" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="D117" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E117" s="11"/>
+      <c r="E117" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F117" s="12">
         <v>39136.0</v>
       </c>
@@ -5168,12 +5401,14 @@
     <row r="118">
       <c r="A118" s="1"/>
       <c r="C118" s="10" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D118" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="E118" s="11"/>
+      <c r="E118" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F118" s="12">
         <v>38666.0</v>
       </c>
@@ -5201,12 +5436,14 @@
     <row r="119">
       <c r="A119" s="1"/>
       <c r="C119" s="10" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>181</v>
-      </c>
-      <c r="E119" s="11"/>
+        <v>183</v>
+      </c>
+      <c r="E119" s="10">
+        <v>69.0</v>
+      </c>
       <c r="F119" s="12">
         <v>39164.0</v>
       </c>
@@ -5234,12 +5471,14 @@
     <row r="120">
       <c r="A120" s="1"/>
       <c r="C120" s="10" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>207</v>
-      </c>
-      <c r="E120" s="11"/>
+        <v>209</v>
+      </c>
+      <c r="E120" s="10">
+        <v>3.0</v>
+      </c>
       <c r="F120" s="12">
         <v>38964.0</v>
       </c>
@@ -5267,16 +5506,18 @@
     <row r="121">
       <c r="A121" s="1"/>
       <c r="B121" s="6" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="D121" s="6" t="s">
-        <v>210</v>
-      </c>
-      <c r="E121" s="6"/>
-      <c r="F121" s="8">
+        <v>212</v>
+      </c>
+      <c r="E121" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F121" s="7">
         <v>36110.0</v>
       </c>
       <c r="G121" s="1"/>
@@ -5308,8 +5549,10 @@
       <c r="D122" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E122" s="6"/>
-      <c r="F122" s="8">
+      <c r="E122" s="6">
+        <v>12.0</v>
+      </c>
+      <c r="F122" s="7">
         <v>33738.0</v>
       </c>
       <c r="G122" s="1"/>
@@ -5336,13 +5579,15 @@
     <row r="123">
       <c r="A123" s="1"/>
       <c r="C123" s="6" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="D123" s="6" t="s">
-        <v>212</v>
-      </c>
-      <c r="E123" s="6"/>
-      <c r="F123" s="8">
+        <v>214</v>
+      </c>
+      <c r="E123" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F123" s="7">
         <v>36453.0</v>
       </c>
       <c r="G123" s="1"/>
@@ -5369,13 +5614,15 @@
     <row r="124">
       <c r="A124" s="1"/>
       <c r="C124" s="6" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="D124" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="E124" s="6"/>
-      <c r="F124" s="8">
+      <c r="E124" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F124" s="7">
         <v>35515.0</v>
       </c>
       <c r="G124" s="1"/>
@@ -5402,13 +5649,15 @@
     <row r="125">
       <c r="A125" s="1"/>
       <c r="C125" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D125" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E125" s="6"/>
-      <c r="F125" s="8">
+      <c r="E125" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F125" s="7">
         <v>34451.0</v>
       </c>
       <c r="G125" s="1"/>
@@ -5435,13 +5684,15 @@
     <row r="126">
       <c r="A126" s="1"/>
       <c r="C126" s="6" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D126" s="6" t="s">
-        <v>216</v>
-      </c>
-      <c r="E126" s="6"/>
-      <c r="F126" s="8">
+        <v>218</v>
+      </c>
+      <c r="E126" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F126" s="7">
         <v>37942.0</v>
       </c>
       <c r="G126" s="1"/>
@@ -5468,13 +5719,15 @@
     <row r="127">
       <c r="A127" s="1"/>
       <c r="C127" s="6" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="D127" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="E127" s="6"/>
-      <c r="F127" s="8">
+      <c r="E127" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F127" s="7">
         <v>37636.0</v>
       </c>
       <c r="G127" s="1"/>
@@ -5506,8 +5759,10 @@
       <c r="D128" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E128" s="6"/>
-      <c r="F128" s="8">
+      <c r="E128" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="F128" s="7">
         <v>39029.0</v>
       </c>
       <c r="G128" s="1"/>
@@ -5534,13 +5789,15 @@
     <row r="129">
       <c r="A129" s="1"/>
       <c r="C129" s="6" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D129" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="E129" s="6"/>
-      <c r="F129" s="8">
+      <c r="E129" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F129" s="7">
         <v>33764.0</v>
       </c>
       <c r="G129" s="1"/>
@@ -5567,15 +5824,17 @@
     <row r="130">
       <c r="A130" s="1"/>
       <c r="B130" s="10" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="C130" s="10" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="D130" s="10" t="s">
-        <v>221</v>
-      </c>
-      <c r="E130" s="11"/>
+        <v>223</v>
+      </c>
+      <c r="E130" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F130" s="12">
         <v>34326.0</v>
       </c>
@@ -5603,12 +5862,14 @@
     <row r="131">
       <c r="A131" s="1"/>
       <c r="C131" s="10" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>223</v>
-      </c>
-      <c r="E131" s="11"/>
+        <v>225</v>
+      </c>
+      <c r="E131" s="10">
+        <v>2.0</v>
+      </c>
       <c r="F131" s="12">
         <v>30482.0</v>
       </c>
@@ -5636,12 +5897,14 @@
     <row r="132">
       <c r="A132" s="1"/>
       <c r="C132" s="10" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="D132" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E132" s="11"/>
+      <c r="E132" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F132" s="12">
         <v>33653.0</v>
       </c>
@@ -5669,12 +5932,14 @@
     <row r="133">
       <c r="A133" s="1"/>
       <c r="C133" s="10" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="D133" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="E133" s="11"/>
+      <c r="E133" s="10">
+        <v>4.0</v>
+      </c>
       <c r="F133" s="12">
         <v>33733.0</v>
       </c>
@@ -5702,12 +5967,14 @@
     <row r="134">
       <c r="A134" s="1"/>
       <c r="C134" s="10" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="E134" s="11"/>
+        <v>229</v>
+      </c>
+      <c r="E134" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F134" s="12">
         <v>35835.0</v>
       </c>
@@ -5735,12 +6002,14 @@
     <row r="135">
       <c r="A135" s="1"/>
       <c r="C135" s="10" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D135" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E135" s="11"/>
+      <c r="E135" s="10">
+        <v>3.0</v>
+      </c>
       <c r="F135" s="12">
         <v>32832.0</v>
       </c>
@@ -5768,12 +6037,14 @@
     <row r="136">
       <c r="A136" s="1"/>
       <c r="C136" s="10" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="D136" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E136" s="11"/>
+      <c r="E136" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F136" s="12">
         <v>38889.0</v>
       </c>
@@ -5801,12 +6072,14 @@
     <row r="137">
       <c r="A137" s="1"/>
       <c r="C137" s="10" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="D137" s="10" t="s">
-        <v>231</v>
-      </c>
-      <c r="E137" s="11"/>
+        <v>233</v>
+      </c>
+      <c r="E137" s="10">
+        <v>7.0</v>
+      </c>
       <c r="F137" s="12">
         <v>34813.0</v>
       </c>
@@ -5834,12 +6107,14 @@
     <row r="138">
       <c r="A138" s="1"/>
       <c r="C138" s="10" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D138" s="10" t="s">
-        <v>233</v>
-      </c>
-      <c r="E138" s="11"/>
+        <v>235</v>
+      </c>
+      <c r="E138" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F138" s="12">
         <v>33864.0</v>
       </c>
@@ -5867,16 +6142,18 @@
     <row r="139">
       <c r="A139" s="1"/>
       <c r="B139" s="6" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="C139" s="6" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D139" s="6" t="s">
-        <v>227</v>
-      </c>
-      <c r="E139" s="6"/>
-      <c r="F139" s="8">
+        <v>238</v>
+      </c>
+      <c r="E139" s="6">
+        <v>22.0</v>
+      </c>
+      <c r="F139" s="7">
         <v>38560.0</v>
       </c>
       <c r="G139" s="1"/>
@@ -5903,13 +6180,15 @@
     <row r="140">
       <c r="A140" s="1"/>
       <c r="C140" s="6" t="s">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="D140" s="6" t="s">
-        <v>233</v>
-      </c>
-      <c r="E140" s="6"/>
-      <c r="F140" s="8">
+        <v>235</v>
+      </c>
+      <c r="E140" s="6">
+        <v>13.0</v>
+      </c>
+      <c r="F140" s="7">
         <v>38897.0</v>
       </c>
       <c r="G140" s="1"/>
@@ -5936,13 +6215,15 @@
     <row r="141">
       <c r="A141" s="1"/>
       <c r="C141" s="6" t="s">
-        <v>237</v>
+        <v>240</v>
       </c>
       <c r="D141" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E141" s="6"/>
-      <c r="F141" s="8">
+      <c r="E141" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="F141" s="7">
         <v>38536.0</v>
       </c>
       <c r="G141" s="1"/>
@@ -5969,13 +6250,15 @@
     <row r="142">
       <c r="A142" s="1"/>
       <c r="C142" s="6" t="s">
-        <v>238</v>
+        <v>241</v>
       </c>
       <c r="D142" s="6" t="s">
-        <v>239</v>
-      </c>
-      <c r="E142" s="6"/>
-      <c r="F142" s="8">
+        <v>242</v>
+      </c>
+      <c r="E142" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F142" s="7">
         <v>40260.0</v>
       </c>
       <c r="G142" s="1"/>
@@ -6002,13 +6285,15 @@
     <row r="143">
       <c r="A143" s="1"/>
       <c r="C143" s="6" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="D143" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E143" s="6"/>
-      <c r="F143" s="8">
+      <c r="E143" s="6">
+        <v>21.0</v>
+      </c>
+      <c r="F143" s="7">
         <v>39521.0</v>
       </c>
       <c r="G143" s="1"/>
@@ -6035,13 +6320,15 @@
     <row r="144">
       <c r="A144" s="1"/>
       <c r="C144" s="6" t="s">
-        <v>241</v>
+        <v>244</v>
       </c>
       <c r="D144" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="E144" s="6"/>
-      <c r="F144" s="8">
+      <c r="E144" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F144" s="7">
         <v>39647.0</v>
       </c>
       <c r="G144" s="1"/>
@@ -6068,13 +6355,15 @@
     <row r="145">
       <c r="A145" s="1"/>
       <c r="C145" s="6" t="s">
-        <v>242</v>
+        <v>245</v>
       </c>
       <c r="D145" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E145" s="6"/>
-      <c r="F145" s="8">
+      <c r="E145" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F145" s="7">
         <v>39547.0</v>
       </c>
       <c r="G145" s="1"/>
@@ -6101,13 +6390,13 @@
     <row r="146">
       <c r="A146" s="1"/>
       <c r="C146" s="6" t="s">
-        <v>243</v>
+        <v>246</v>
       </c>
       <c r="D146" s="6" t="s">
-        <v>244</v>
+        <v>247</v>
       </c>
       <c r="E146" s="6"/>
-      <c r="F146" s="8">
+      <c r="F146" s="7">
         <v>39730.0</v>
       </c>
       <c r="G146" s="1"/>
@@ -6134,15 +6423,17 @@
     <row r="147">
       <c r="A147" s="1"/>
       <c r="B147" s="10" t="s">
-        <v>245</v>
+        <v>248</v>
       </c>
       <c r="C147" s="10" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D147" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="E147" s="11"/>
+      <c r="E147" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F147" s="12">
         <v>38520.0</v>
       </c>
@@ -6173,9 +6464,11 @@
         <v>175</v>
       </c>
       <c r="D148" s="10" t="s">
-        <v>227</v>
-      </c>
-      <c r="E148" s="11"/>
+        <v>238</v>
+      </c>
+      <c r="E148" s="10">
+        <v>87.0</v>
+      </c>
       <c r="F148" s="12">
         <v>37705.0</v>
       </c>
@@ -6208,7 +6501,9 @@
       <c r="D149" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E149" s="11"/>
+      <c r="E149" s="10">
+        <v>11.0</v>
+      </c>
       <c r="F149" s="12">
         <v>38524.0</v>
       </c>
@@ -6241,7 +6536,9 @@
       <c r="D150" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E150" s="11"/>
+      <c r="E150" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F150" s="12">
         <v>39106.0</v>
       </c>
@@ -6269,12 +6566,14 @@
     <row r="151">
       <c r="A151" s="1"/>
       <c r="C151" s="10" t="s">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="D151" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="E151" s="11"/>
+      <c r="E151" s="10">
+        <v>7.0</v>
+      </c>
       <c r="F151" s="12">
         <v>37666.0</v>
       </c>
@@ -6302,12 +6601,14 @@
     <row r="152">
       <c r="A152" s="1"/>
       <c r="C152" s="10" t="s">
-        <v>248</v>
+        <v>251</v>
       </c>
       <c r="D152" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="E152" s="11"/>
+      <c r="E152" s="10">
+        <v>22.0</v>
+      </c>
       <c r="F152" s="12">
         <v>37720.0</v>
       </c>
@@ -6335,12 +6636,14 @@
     <row r="153">
       <c r="A153" s="1"/>
       <c r="C153" s="10" t="s">
-        <v>249</v>
+        <v>252</v>
       </c>
       <c r="D153" s="10" t="s">
-        <v>250</v>
-      </c>
-      <c r="E153" s="11"/>
+        <v>253</v>
+      </c>
+      <c r="E153" s="10">
+        <v>4.0</v>
+      </c>
       <c r="F153" s="12">
         <v>38048.0</v>
       </c>
@@ -6368,12 +6671,14 @@
     <row r="154">
       <c r="A154" s="1"/>
       <c r="C154" s="10" t="s">
-        <v>251</v>
+        <v>254</v>
       </c>
       <c r="D154" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E154" s="11"/>
+      <c r="E154" s="10">
+        <v>88.0</v>
+      </c>
       <c r="F154" s="12">
         <v>35535.0</v>
       </c>
@@ -6401,12 +6706,14 @@
     <row r="155">
       <c r="A155" s="1"/>
       <c r="C155" s="10" t="s">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="D155" s="10" t="s">
-        <v>253</v>
-      </c>
-      <c r="E155" s="11"/>
+        <v>256</v>
+      </c>
+      <c r="E155" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F155" s="12">
         <v>37826.0</v>
       </c>
@@ -6434,12 +6741,14 @@
     <row r="156">
       <c r="A156" s="1"/>
       <c r="C156" s="10" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="D156" s="10" t="s">
-        <v>255</v>
-      </c>
-      <c r="E156" s="10"/>
+        <v>258</v>
+      </c>
+      <c r="E156" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F156" s="12">
         <v>33544.0</v>
       </c>
@@ -6467,12 +6776,14 @@
     <row r="157">
       <c r="A157" s="1"/>
       <c r="C157" s="10" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="D157" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E157" s="11"/>
+      <c r="E157" s="10">
+        <v>2.0</v>
+      </c>
       <c r="F157" s="12">
         <v>36748.0</v>
       </c>
@@ -6500,16 +6811,18 @@
     <row r="158">
       <c r="A158" s="1"/>
       <c r="B158" s="6" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="C158" s="6" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
       <c r="D158" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="E158" s="6"/>
-      <c r="F158" s="8">
+      <c r="E158" s="6">
+        <v>7.0</v>
+      </c>
+      <c r="F158" s="7">
         <v>35167.0</v>
       </c>
       <c r="G158" s="1"/>
@@ -6536,13 +6849,15 @@
     <row r="159">
       <c r="A159" s="1"/>
       <c r="C159" s="6" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
       <c r="D159" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="E159" s="6"/>
-      <c r="F159" s="8">
+      <c r="E159" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F159" s="7">
         <v>35393.0</v>
       </c>
       <c r="G159" s="1"/>
@@ -6574,8 +6889,10 @@
       <c r="D160" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="E160" s="6"/>
-      <c r="F160" s="8">
+      <c r="E160" s="6">
+        <v>3.0</v>
+      </c>
+      <c r="F160" s="7">
         <v>35329.0</v>
       </c>
       <c r="G160" s="1"/>
@@ -6602,13 +6919,15 @@
     <row r="161">
       <c r="A161" s="1"/>
       <c r="C161" s="6" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="D161" s="6" t="s">
-        <v>261</v>
-      </c>
-      <c r="E161" s="6"/>
-      <c r="F161" s="8">
+        <v>264</v>
+      </c>
+      <c r="E161" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F161" s="7">
         <v>36457.0</v>
       </c>
       <c r="G161" s="1"/>
@@ -6635,13 +6954,15 @@
     <row r="162">
       <c r="A162" s="1"/>
       <c r="C162" s="6" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="D162" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E162" s="6"/>
-      <c r="F162" s="8">
+      <c r="E162" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F162" s="7">
         <v>36945.0</v>
       </c>
       <c r="G162" s="1"/>
@@ -6668,13 +6989,15 @@
     <row r="163">
       <c r="A163" s="1"/>
       <c r="C163" s="6" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="D163" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E163" s="6"/>
-      <c r="F163" s="8">
+      <c r="E163" s="6">
+        <v>4.0</v>
+      </c>
+      <c r="F163" s="7">
         <v>36836.0</v>
       </c>
       <c r="G163" s="1"/>
@@ -6701,13 +7024,15 @@
     <row r="164">
       <c r="A164" s="1"/>
       <c r="C164" s="6" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="D164" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="E164" s="6"/>
-      <c r="F164" s="8">
+      <c r="E164" s="6">
+        <v>16.0</v>
+      </c>
+      <c r="F164" s="7">
         <v>30572.0</v>
       </c>
       <c r="G164" s="1"/>
@@ -6734,13 +7059,15 @@
     <row r="165">
       <c r="A165" s="1"/>
       <c r="C165" s="6" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="D165" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="E165" s="6"/>
-      <c r="F165" s="8">
+      <c r="E165" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F165" s="7">
         <v>36169.0</v>
       </c>
       <c r="G165" s="1"/>
@@ -6767,17 +7094,19 @@
     <row r="166">
       <c r="A166" s="1"/>
       <c r="B166" s="10" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="C166" s="10" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="D166" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="E166" s="11"/>
+      <c r="E166" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F166" s="12" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="G166" s="1"/>
       <c r="H166" s="1"/>
@@ -6803,14 +7132,16 @@
     <row r="167">
       <c r="A167" s="1"/>
       <c r="C167" s="10" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="D167" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="E167" s="11"/>
+      <c r="E167" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F167" s="12" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="G167" s="1"/>
       <c r="H167" s="1"/>
@@ -6836,14 +7167,16 @@
     <row r="168">
       <c r="A168" s="1"/>
       <c r="C168" s="10" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D168" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="E168" s="11"/>
+      <c r="E168" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F168" s="12" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="G168" s="1"/>
       <c r="H168" s="1"/>
@@ -6869,14 +7202,16 @@
     <row r="169">
       <c r="A169" s="1"/>
       <c r="C169" s="10" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="D169" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="E169" s="11"/>
+      <c r="E169" s="10">
+        <v>77.0</v>
+      </c>
       <c r="F169" s="12" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="G169" s="1"/>
       <c r="H169" s="1"/>
@@ -6902,14 +7237,16 @@
     <row r="170">
       <c r="A170" s="1"/>
       <c r="C170" s="10" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="D170" s="10" t="s">
-        <v>276</v>
-      </c>
-      <c r="E170" s="11"/>
+        <v>279</v>
+      </c>
+      <c r="E170" s="10">
+        <v>5.0</v>
+      </c>
       <c r="F170" s="12" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="G170" s="1"/>
       <c r="H170" s="1"/>
@@ -6935,14 +7272,16 @@
     <row r="171">
       <c r="A171" s="1"/>
       <c r="C171" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D171" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="E171" s="11"/>
+      <c r="E171" s="10">
+        <v>69.0</v>
+      </c>
       <c r="F171" s="12" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="G171" s="1"/>
       <c r="H171" s="1"/>
@@ -6968,14 +7307,16 @@
     <row r="172">
       <c r="A172" s="1"/>
       <c r="C172" s="10" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="D172" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="E172" s="11"/>
+        <v>284</v>
+      </c>
+      <c r="E172" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F172" s="12" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="G172" s="1"/>
       <c r="H172" s="1"/>
@@ -7001,14 +7342,16 @@
     <row r="173">
       <c r="A173" s="1"/>
       <c r="C173" s="10" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="D173" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E173" s="11"/>
+      <c r="E173" s="10">
+        <v>45.0</v>
+      </c>
       <c r="F173" s="12" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="G173" s="1"/>
       <c r="H173" s="1"/>
@@ -7034,14 +7377,16 @@
     <row r="174">
       <c r="A174" s="1"/>
       <c r="C174" s="10" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="D174" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="E174" s="11"/>
+      <c r="E174" s="10">
+        <v>21.0</v>
+      </c>
       <c r="F174" s="12" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="G174" s="1"/>
       <c r="H174" s="1"/>
@@ -7067,16 +7412,18 @@
     <row r="175">
       <c r="A175" s="1"/>
       <c r="B175" s="6" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="C175" s="6" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="D175" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E175" s="6"/>
-      <c r="F175" s="8">
+      <c r="E175" s="6">
+        <v>14.0</v>
+      </c>
+      <c r="F175" s="7">
         <v>38052.0</v>
       </c>
       <c r="G175" s="1"/>
@@ -7103,13 +7450,15 @@
     <row r="176">
       <c r="A176" s="1"/>
       <c r="C176" s="6" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="D176" s="6" t="s">
-        <v>290</v>
-      </c>
-      <c r="E176" s="6"/>
-      <c r="F176" s="8">
+        <v>293</v>
+      </c>
+      <c r="E176" s="6">
+        <v>22.0</v>
+      </c>
+      <c r="F176" s="7">
         <v>37297.0</v>
       </c>
       <c r="G176" s="1"/>
@@ -7136,13 +7485,15 @@
     <row r="177">
       <c r="A177" s="1"/>
       <c r="C177" s="6" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D177" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="E177" s="6"/>
-      <c r="F177" s="8">
+      <c r="E177" s="6">
+        <v>8.0</v>
+      </c>
+      <c r="F177" s="7">
         <v>38253.0</v>
       </c>
       <c r="G177" s="1"/>
@@ -7169,13 +7520,15 @@
     <row r="178">
       <c r="A178" s="1"/>
       <c r="C178" s="6" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="D178" s="6" t="s">
-        <v>292</v>
-      </c>
-      <c r="E178" s="6"/>
-      <c r="F178" s="8">
+        <v>295</v>
+      </c>
+      <c r="E178" s="6">
+        <v>6.0</v>
+      </c>
+      <c r="F178" s="7">
         <v>38869.0</v>
       </c>
       <c r="G178" s="1"/>
@@ -7202,13 +7555,15 @@
     <row r="179">
       <c r="A179" s="1"/>
       <c r="C179" s="6" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="D179" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E179" s="6"/>
-      <c r="F179" s="8">
+      <c r="E179" s="6">
+        <v>11.0</v>
+      </c>
+      <c r="F179" s="7">
         <v>38890.0</v>
       </c>
       <c r="G179" s="1"/>
@@ -7235,13 +7590,15 @@
     <row r="180">
       <c r="A180" s="1"/>
       <c r="C180" s="6" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="D180" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="E180" s="6"/>
-      <c r="F180" s="8">
+      <c r="E180" s="6">
+        <v>1.0</v>
+      </c>
+      <c r="F180" s="7">
         <v>38809.0</v>
       </c>
       <c r="G180" s="1"/>
@@ -7268,13 +7625,15 @@
     <row r="181">
       <c r="A181" s="1"/>
       <c r="C181" s="6" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D181" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="E181" s="6"/>
-      <c r="F181" s="8">
+      <c r="E181" s="6">
+        <v>5.0</v>
+      </c>
+      <c r="F181" s="7">
         <v>38046.0</v>
       </c>
       <c r="G181" s="1"/>
@@ -7301,13 +7660,15 @@
     <row r="182">
       <c r="A182" s="1"/>
       <c r="C182" s="6" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="D182" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="E182" s="6"/>
-      <c r="F182" s="8">
+      <c r="E182" s="6">
+        <v>9.0</v>
+      </c>
+      <c r="F182" s="7">
         <v>38054.0</v>
       </c>
       <c r="G182" s="1"/>
@@ -7334,13 +7695,15 @@
     <row r="183">
       <c r="A183" s="1"/>
       <c r="C183" s="6" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D183" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="E183" s="6"/>
-      <c r="F183" s="8">
+      <c r="E183" s="6">
+        <v>2.0</v>
+      </c>
+      <c r="F183" s="7">
         <v>38956.0</v>
       </c>
       <c r="G183" s="1"/>
@@ -7367,13 +7730,15 @@
     <row r="184">
       <c r="A184" s="1"/>
       <c r="C184" s="6" t="s">
-        <v>246</v>
+        <v>249</v>
       </c>
       <c r="D184" s="6" t="s">
-        <v>297</v>
-      </c>
-      <c r="E184" s="6"/>
-      <c r="F184" s="8">
+        <v>300</v>
+      </c>
+      <c r="E184" s="6">
+        <v>10.0</v>
+      </c>
+      <c r="F184" s="7">
         <v>38920.0</v>
       </c>
       <c r="G184" s="1"/>
@@ -7400,15 +7765,17 @@
     <row r="185">
       <c r="A185" s="1"/>
       <c r="B185" s="10" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="C185" s="10" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="D185" s="10" t="s">
-        <v>179</v>
-      </c>
-      <c r="E185" s="11"/>
+        <v>181</v>
+      </c>
+      <c r="E185" s="10">
+        <v>1.0</v>
+      </c>
       <c r="F185" s="12">
         <v>39255.0</v>
       </c>
@@ -7436,12 +7803,14 @@
     <row r="186">
       <c r="A186" s="1"/>
       <c r="C186" s="10" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="D186" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="E186" s="11"/>
+      <c r="E186" s="10">
+        <v>9.0</v>
+      </c>
       <c r="F186" s="12">
         <v>37346.0</v>
       </c>
@@ -7469,12 +7838,14 @@
     <row r="187">
       <c r="A187" s="1"/>
       <c r="C187" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D187" s="10" t="s">
-        <v>302</v>
-      </c>
-      <c r="E187" s="11"/>
+        <v>305</v>
+      </c>
+      <c r="E187" s="10">
+        <v>17.0</v>
+      </c>
       <c r="F187" s="12">
         <v>39730.0</v>
       </c>
@@ -7502,12 +7873,14 @@
     <row r="188">
       <c r="A188" s="1"/>
       <c r="C188" s="10" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="D188" s="10" t="s">
-        <v>304</v>
-      </c>
-      <c r="E188" s="11"/>
+        <v>307</v>
+      </c>
+      <c r="E188" s="10">
+        <v>6.0</v>
+      </c>
       <c r="F188" s="12">
         <v>39786.0</v>
       </c>
@@ -7535,12 +7908,14 @@
     <row r="189">
       <c r="A189" s="1"/>
       <c r="C189" s="10" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="D189" s="10" t="s">
-        <v>306</v>
-      </c>
-      <c r="E189" s="11"/>
+        <v>309</v>
+      </c>
+      <c r="E189" s="10">
+        <v>10.0</v>
+      </c>
       <c r="F189" s="12">
         <v>38635.0</v>
       </c>
@@ -7568,12 +7943,14 @@
     <row r="190">
       <c r="A190" s="1"/>
       <c r="C190" s="10" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="D190" s="10" t="s">
-        <v>308</v>
-      </c>
-      <c r="E190" s="11"/>
+        <v>311</v>
+      </c>
+      <c r="E190" s="10">
+        <v>11.0</v>
+      </c>
       <c r="F190" s="12">
         <v>38576.0</v>
       </c>
@@ -7601,12 +7978,14 @@
     <row r="191">
       <c r="A191" s="1"/>
       <c r="C191" s="10" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D191" s="10" t="s">
-        <v>310</v>
-      </c>
-      <c r="E191" s="11"/>
+        <v>313</v>
+      </c>
+      <c r="E191" s="10">
+        <v>8.0</v>
+      </c>
       <c r="F191" s="12">
         <v>38605.0</v>
       </c>
@@ -7634,12 +8013,14 @@
     <row r="192">
       <c r="A192" s="1"/>
       <c r="C192" s="10" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="D192" s="10" t="s">
-        <v>312</v>
-      </c>
-      <c r="E192" s="11"/>
+        <v>315</v>
+      </c>
+      <c r="E192" s="10">
+        <v>47.0</v>
+      </c>
       <c r="F192" s="12">
         <v>39041.0</v>
       </c>

</xml_diff>